<commit_message>
fix(finance): canonical_division_code -- close the 1012-vs-10-12 division trap
Filenames spell range divisions dashless (settled convention: a dash
collides with the naming separators); the DB canonical form is the dash
range. The Phase 5 quote-document resolver exact-matched the raw filename
code against SowPackage.division_code, so a range-division quote (e.g.
Fixtures) could never resolve its package -- found while auditing, before
any real quote hit it.

financial_divisions.canonical_division_code() folds dashless 4-digit and
single range members to canonical ("1012"/"10"/"11"/"12" -> "10-12"),
passes canonical codes through, and leaves unknowns unchanged so callers
flag rather than lose them. Applied at the resolver parse boundary.
Template generator cells canonicalized to "10-12" (filenames stay
dashless via csi.replace); mock Drive regenerated. 2 new parse cases.

Suite: 1676 passed.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/templates/mock_drive/2026001 — Rockland/SOW/2026001_SOW_v1.xlsx
+++ b/docs/templates/mock_drive/2026001 — Rockland/SOW/2026001_SOW_v1.xlsx
@@ -1219,7 +1219,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>1012</t>
+          <t>10-12</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>1012</t>
+          <t>10-12</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>1012</t>
+          <t>10-12</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">

</xml_diff>